<commit_message>
Add Deposit Amount column to Customer Bulk Import format and customer schema
</commit_message>
<xml_diff>
--- a/public/templates/Customer_Template.xlsx
+++ b/public/templates/Customer_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>InitialBalance</v>
       </c>
+      <c r="E1" t="str">
+        <v>DepositAmount</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,6 +429,9 @@
       <c r="D2">
         <v>50</v>
       </c>
+      <c r="E2">
+        <v>100000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,10 +446,13 @@
       <c r="D3">
         <v>0</v>
       </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>